<commit_message>
add baostock csi300 downloader
</commit_message>
<xml_diff>
--- a/docs/notes/result.xlsx
+++ b/docs/notes/result.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kc/Development/qlib/qlib/docs/notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F234A1-0157-1D43-97E5-3B94BF6D54CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{791EE10B-0BAE-0E4A-8294-F2CC16B7BD27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10240" yWindow="23160" windowWidth="28040" windowHeight="17440" xr2:uid="{927EE297-4ED8-F044-B20F-C4461B5F7F44}"/>
+    <workbookView xWindow="6340" yWindow="23780" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{927EE297-4ED8-F044-B20F-C4461B5F7F44}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="训练到 2019 年底" sheetId="1" r:id="rId1"/>
+    <sheet name="训练到 2020 年底" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
   <si>
     <t>paper:</t>
   </si>
@@ -176,6 +177,67 @@
   </si>
   <si>
     <t>四年总收益:-6.28%</t>
+  </si>
+  <si>
+    <t>train: [2008-01-01, 2020-12-31]
+valid: [2021-01-01, 2022-12-31]
+test: [2024-01-01, 2024-12-31]</t>
+  </si>
+  <si>
+    <t>train: [2008-01-01, 2020-12-31]
+valid: [2021-01-01, 2022-12-31]
+test: [2023-01-01, 2023-12-31]</t>
+  </si>
+  <si>
+    <t>train: [2008-01-01, 2020-12-31]
+valid: [2021-01-01, 2022-12-31]
+test: [2025-01-01, 2025-12-31]</t>
+  </si>
+  <si>
+    <t>train: [2008-01-01, 2020-12-31]
+valid: [2021-01-01, 2022-12-31]
+test: [2023-01-01, 2025-12-31]</t>
+  </si>
+  <si>
+    <t>mean               0.000466
+std                0.009505
+annualized_return  0.110852
+information_ratio  0.755993
+max_drawdown      -0.173672</t>
+  </si>
+  <si>
+    <t>mean               0.000722
+std                0.010602
+annualized_return  0.171786
+information_ratio  1.050269
+max_drawdown      -0.120876</t>
+  </si>
+  <si>
+    <t>train: [2008-01-01, 2019-12-31]
+valid: [2020-01-01, 2021-12-31]
+test: [2023-01-01, 2025-12-31]</t>
+  </si>
+  <si>
+    <t>mean               0.000229
+std                0.009259
+annualized_return  0.054468
+information_ratio  0.381329
+max_drawdown      -0.142983</t>
+  </si>
+  <si>
+    <t>mean               0.000642
+std                0.008056
+annualized_return  0.152722
+information_ratio  1.228902
+max_drawdown      -0.078697</t>
+  </si>
+  <si>
+    <t>和市场对比</t>
+  </si>
+  <si>
+    <t>沪深 300 为 19.59%
+幻方的三年总收益应该是有 80%+
+我们三年下来月增长 120%</t>
   </si>
 </sst>
 </file>
@@ -556,7 +618,7 @@
     <col min="1" max="1" width="48.1640625" customWidth="1"/>
     <col min="2" max="2" width="27.5" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -570,7 +632,7 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="88" customHeight="1" x14ac:dyDescent="0.2">
@@ -645,7 +707,7 @@
     </row>
     <row r="10" spans="1:4" ht="85" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>24</v>
@@ -654,6 +716,92 @@
         <v>25</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7019F658-15B9-CC45-BC0D-BC0018B8871F}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="33" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="85" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>